<commit_message>
correct bundle discriminator (#67) d07f42af6e84eeaf63a448029d3e8a8bd33c0c83
</commit_message>
<xml_diff>
--- a/ig/main/StructureDefinition-mesures-bundle-flux-alimentation.xlsx
+++ b/ig/main/StructureDefinition-mesures-bundle-flux-alimentation.xlsx
@@ -54,7 +54,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-09-20T15:08:45+00:00</t>
+    <t>2023-09-27T13:54:59+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -473,11 +473,11 @@
     <t>An entry in a bundle resource - will either contain a resource or information about a resource (transactions and history only).</t>
   </si>
   <si>
-    <t xml:space="preserve">pattern:entry.request.url}
+    <t xml:space="preserve">profile:request.url}
 </t>
   </si>
   <si>
-    <t>Slice based on the entry.request.url pattern</t>
+    <t>Slice based on the request.url pattern</t>
   </si>
   <si>
     <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
@@ -1340,7 +1340,7 @@
     <col min="25" max="25" width="168.19140625" customWidth="true" bestFit="true"/>
     <col min="26" max="26" width="49.01171875" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="1.04296875" customWidth="true" bestFit="true"/>
-    <col min="28" max="28" width="25.04296875" customWidth="true" bestFit="true"/>
+    <col min="28" max="28" width="18.67578125" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="42.03515625" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="1.04296875" customWidth="true" bestFit="true"/>
     <col min="31" max="31" width="5.62109375" customWidth="true" bestFit="true" hidden="true"/>

</xml_diff>

<commit_message>
Correction du Q/A et résolution des erreurs des exemples (#99)
* resolve errors

* resolve example error 6681eb2658e0b4eaf7e73d1f851e321433c16fcb
</commit_message>
<xml_diff>
--- a/ig/main/StructureDefinition-mesures-bundle-flux-alimentation.xlsx
+++ b/ig/main/StructureDefinition-mesures-bundle-flux-alimentation.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-02-01T16:04:25+00:00</t>
+    <t>2024-02-05T14:48:49+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -602,7 +602,7 @@
     <t>An entry in a bundle resource - will either contain a resource or information about a resource (transactions and history only).</t>
   </si>
   <si>
-    <t xml:space="preserve">profile:request.url}
+    <t xml:space="preserve">pattern:request.url}
 </t>
   </si>
   <si>

</xml_diff>